<commit_message>
updated readme + added new libraries seeedpy
</commit_message>
<xml_diff>
--- a/Modbus_protocol/buffer_addresses.xlsx
+++ b/Modbus_protocol/buffer_addresses.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="116" uniqueCount="72">
   <si>
     <t xml:space="preserve">Identification (from doc manual)</t>
   </si>
@@ -164,6 +164,9 @@
   </si>
   <si>
     <t xml:space="preserve">0x0037</t>
+  </si>
+  <si>
+    <t xml:space="preserve">read and write</t>
   </si>
   <si>
     <t xml:space="preserve">0x2001</t>
@@ -436,7 +439,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:I27"/>
-  <sheetFormatPr defaultColWidth="9.2109375" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="9.21875" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="21.87"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="8.33"/>
@@ -835,6 +838,9 @@
       <c r="H15" s="2" t="s">
         <v>12</v>
       </c>
+      <c r="I15" s="0" t="s">
+        <v>48</v>
+      </c>
     </row>
     <row r="16" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="3" t="s">
@@ -842,7 +848,7 @@
       </c>
       <c r="B16" s="3"/>
       <c r="C16" s="4" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="D16" s="4" t="n">
         <v>8193</v>
@@ -854,13 +860,13 @@
         <v>5</v>
       </c>
       <c r="G16" s="4" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="H16" s="4" t="s">
         <v>12</v>
       </c>
       <c r="I16" s="5" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -869,7 +875,7 @@
       </c>
       <c r="B17" s="3"/>
       <c r="C17" s="4" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="D17" s="4" t="n">
         <v>8194</v>
@@ -887,16 +893,16 @@
         <v>12</v>
       </c>
       <c r="I17" s="5" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="3" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B18" s="3"/>
       <c r="C18" s="2" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="D18" s="2" t="n">
         <v>8195</v>
@@ -914,7 +920,7 @@
         <v>12</v>
       </c>
       <c r="I18" s="0" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -923,7 +929,7 @@
       </c>
       <c r="B19" s="3"/>
       <c r="C19" s="4" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D19" s="4" t="n">
         <v>8196</v>
@@ -935,13 +941,13 @@
         <v>2024</v>
       </c>
       <c r="G19" s="4" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="H19" s="4" t="s">
         <v>12</v>
       </c>
       <c r="I19" s="5" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -950,7 +956,7 @@
       </c>
       <c r="B20" s="3"/>
       <c r="C20" s="4" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="D20" s="4" t="n">
         <v>8197</v>
@@ -962,57 +968,57 @@
         <v>304</v>
       </c>
       <c r="G20" s="4" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="H20" s="4" t="s">
         <v>12</v>
       </c>
       <c r="I20" s="5" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="3" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="D21" s="2" t="n">
         <v>8224</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="F21" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="G21" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="H21" s="2" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="I21" s="0" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C24" s="0" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="24.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C26" s="6" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C27" s="5" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
     </row>
   </sheetData>

</xml_diff>